<commit_message>
hopefully the last change
</commit_message>
<xml_diff>
--- a/Post-processing.xlsx
+++ b/Post-processing.xlsx
@@ -469,6 +469,11 @@
       <c r="A2" s="1" t="n">
         <v>0.25</v>
       </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>e</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">

</xml_diff>